<commit_message>
Bringe README auf finalen Stand
</commit_message>
<xml_diff>
--- a/Usability-Test-PT-Karteikarten.xlsx
+++ b/Usability-Test-PT-Karteikarten.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/renato/Desktop/Prototyping/PT Karteikarten/PT-Karteikarten/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EE039C3-3101-4E45-86A1-287D3F3E23F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D56A3C31-8A67-274D-AB4C-208FFA045168}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="37840" windowHeight="20360" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="37840" windowHeight="20360" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Überblick (2)" sheetId="9" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="157">
   <si>
     <t>PT-Karteikarten – Usability Test Tracking</t>
   </si>
@@ -338,9 +338,6 @@
     <t>Du möchtest für ein neues Modul eine eigene Sammlung anlegen und hast ausserdem bemerkt, dass eine Sammlung doppelt vorhanden ist und gelöscht werden soll.</t>
   </si>
   <si>
-    <t>nein</t>
-  </si>
-  <si>
     <t>Ja hat Dashbvoard nicht auf Anhieb gefunden, hat zuerst auf Stapelübersciht geklickt</t>
   </si>
   <si>
@@ -501,6 +498,12 @@
   </si>
   <si>
     <t>Testperson</t>
+  </si>
+  <si>
+    <t>Ja ich wusste nicht wie ich diese einem Stapel zuornden kann oder ob es einen neuen erstellt</t>
+  </si>
+  <si>
+    <t>Einfach war gut so</t>
   </si>
 </sst>
 </file>
@@ -751,33 +754,36 @@
     <xf numFmtId="14" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
@@ -788,6 +794,12 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
@@ -796,15 +808,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -821,104 +824,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>128698</xdr:colOff>
-      <xdr:row>80</xdr:row>
-      <xdr:rowOff>174863</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Grafik 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E3176EAC-8040-3448-A98A-09064C875E45}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="10248900" y="11049000"/>
-          <a:ext cx="6186598" cy="10080863"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>128698</xdr:colOff>
-      <xdr:row>80</xdr:row>
-      <xdr:rowOff>174863</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Grafik 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{691C09E9-F6E9-06B2-4E9E-96CE6808B927}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="10255034" y="10954830"/>
-          <a:ext cx="6193596" cy="10058400"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1219,7 +1124,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="18"/>
@@ -1227,15 +1132,15 @@
       <c r="D1" s="18"/>
     </row>
     <row r="2" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
-        <v>125</v>
+      <c r="A2" s="20" t="s">
+        <v>124</v>
       </c>
       <c r="B2" s="18"/>
       <c r="C2" s="18"/>
       <c r="D2" s="18"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="21" t="s">
         <v>1</v>
       </c>
       <c r="B4" s="18"/>
@@ -1263,7 +1168,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -1271,19 +1176,19 @@
         <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B9" s="2">
         <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="22" t="s">
+      <c r="A10" s="21" t="s">
         <v>7</v>
       </c>
       <c r="B10" s="18"/>
@@ -1291,7 +1196,7 @@
       <c r="D10" s="18"/>
     </row>
     <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="17" t="s">
         <v>8</v>
       </c>
       <c r="B11" s="18"/>
@@ -1299,7 +1204,7 @@
       <c r="D11" s="18"/>
     </row>
     <row r="12" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="17" t="s">
         <v>9</v>
       </c>
       <c r="B12" s="18"/>
@@ -1307,7 +1212,7 @@
       <c r="D12" s="18"/>
     </row>
     <row r="13" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="17" t="s">
         <v>10</v>
       </c>
       <c r="B13" s="18"/>
@@ -1315,7 +1220,7 @@
       <c r="D13" s="18"/>
     </row>
     <row r="14" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="21" t="s">
+      <c r="A14" s="17" t="s">
         <v>11</v>
       </c>
       <c r="B14" s="18"/>
@@ -1323,7 +1228,7 @@
       <c r="D14" s="18"/>
     </row>
     <row r="15" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="21" t="s">
+      <c r="A15" s="17" t="s">
         <v>12</v>
       </c>
       <c r="B15" s="18"/>
@@ -1331,7 +1236,7 @@
       <c r="D15" s="18"/>
     </row>
     <row r="16" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="21" t="s">
+      <c r="A16" s="17" t="s">
         <v>13</v>
       </c>
       <c r="B16" s="18"/>
@@ -1339,7 +1244,7 @@
       <c r="D16" s="18"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="21" t="s">
         <v>14</v>
       </c>
       <c r="B18" s="18"/>
@@ -1431,7 +1336,7 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="22" t="s">
+      <c r="A26" s="21" t="s">
         <v>31</v>
       </c>
       <c r="B26" s="18"/>
@@ -1442,7 +1347,7 @@
       <c r="A27" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B27" s="17" t="s">
+      <c r="B27" s="22" t="s">
         <v>33</v>
       </c>
       <c r="C27" s="18"/>
@@ -1452,7 +1357,7 @@
       <c r="A28" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B28" s="19" t="s">
+      <c r="B28" s="23" t="s">
         <v>35</v>
       </c>
       <c r="C28" s="18"/>
@@ -1462,7 +1367,7 @@
       <c r="A29" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="B29" s="20" t="s">
+      <c r="B29" s="24" t="s">
         <v>37</v>
       </c>
       <c r="C29" s="18"/>
@@ -1470,12 +1375,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A11:D11"/>
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="B28:D28"/>
     <mergeCell ref="B29:D29"/>
@@ -1485,6 +1384,12 @@
     <mergeCell ref="A16:D16"/>
     <mergeCell ref="A18:D18"/>
     <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A11:D11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1503,7 +1408,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>61</v>
       </c>
       <c r="B1" s="18"/>
@@ -1511,7 +1416,7 @@
       <c r="D1" s="18"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>39</v>
       </c>
       <c r="B2" s="18"/>
@@ -1519,15 +1424,15 @@
       <c r="D2" s="18"/>
     </row>
     <row r="3" spans="1:4" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="29" t="s">
-        <v>110</v>
+      <c r="A3" s="30" t="s">
+        <v>109</v>
       </c>
       <c r="B3" s="18"/>
       <c r="C3" s="18"/>
       <c r="D3" s="18"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
         <v>62</v>
       </c>
       <c r="B5" s="18"/>
@@ -1535,7 +1440,7 @@
       <c r="D5" s="18"/>
     </row>
     <row r="6" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="28" t="s">
         <v>63</v>
       </c>
       <c r="B6" s="18"/>
@@ -1546,11 +1451,11 @@
       <c r="A7" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="34"/>
-      <c r="D7" s="35"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="27"/>
     </row>
     <row r="8" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
@@ -1569,7 +1474,9 @@
       <c r="B9" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="4"/>
+      <c r="C9" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D9" s="4"/>
     </row>
     <row r="10" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
@@ -1579,11 +1486,13 @@
       <c r="B10" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="4"/>
+      <c r="C10" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D10" s="4"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="31" t="s">
         <v>64</v>
       </c>
       <c r="B11" s="18"/>
@@ -1594,11 +1503,11 @@
       <c r="A12" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B12" s="32" t="s">
+      <c r="B12" s="35" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="26" t="s">
-        <v>112</v>
+      <c r="C12" s="32" t="s">
+        <v>111</v>
       </c>
       <c r="D12" s="18"/>
     </row>
@@ -1606,10 +1515,10 @@
       <c r="A13" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B13" s="32" t="s">
+      <c r="B13" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="31" t="s">
+      <c r="C13" s="34" t="s">
         <v>36</v>
       </c>
       <c r="D13" s="18"/>
@@ -1618,11 +1527,11 @@
       <c r="A14" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B14" s="32" t="s">
+      <c r="B14" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="26" t="s">
-        <v>111</v>
+      <c r="C14" s="32" t="s">
+        <v>110</v>
       </c>
       <c r="D14" s="18"/>
     </row>
@@ -1630,16 +1539,23 @@
       <c r="A15" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B15" s="32" t="s">
+      <c r="B15" s="35" t="s">
         <v>57</v>
       </c>
-      <c r="C15" s="31" t="s">
+      <c r="C15" s="34" t="s">
         <v>32</v>
       </c>
       <c r="D15" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="B14"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="B15"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="B13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A6:D6"/>
@@ -1648,13 +1564,6 @@
     <mergeCell ref="A11:D11"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="B7:D7"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="B14"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="B15"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="B13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1673,7 +1582,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>65</v>
       </c>
       <c r="B1" s="18"/>
@@ -1681,7 +1590,7 @@
       <c r="D1" s="18"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>39</v>
       </c>
       <c r="B2" s="18"/>
@@ -1689,7 +1598,7 @@
       <c r="D2" s="18"/>
     </row>
     <row r="3" spans="1:4" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="30" t="s">
+      <c r="A3" s="33" t="s">
         <v>100</v>
       </c>
       <c r="B3" s="18"/>
@@ -1697,7 +1606,7 @@
       <c r="D3" s="18"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
         <v>66</v>
       </c>
       <c r="B5" s="18"/>
@@ -1705,7 +1614,7 @@
       <c r="D5" s="18"/>
     </row>
     <row r="6" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="28" t="s">
         <v>67</v>
       </c>
       <c r="B6" s="18"/>
@@ -1716,11 +1625,11 @@
       <c r="A7" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="34"/>
-      <c r="D7" s="35"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="27"/>
     </row>
     <row r="8" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
@@ -1729,7 +1638,9 @@
       <c r="B8" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="4"/>
+      <c r="C8" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D8" s="4"/>
     </row>
     <row r="9" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
@@ -1739,7 +1650,9 @@
       <c r="B9" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="4"/>
+      <c r="C9" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D9" s="4"/>
     </row>
     <row r="10" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
@@ -1749,11 +1662,13 @@
       <c r="B10" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="4"/>
+      <c r="C10" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D10" s="4"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="31" t="s">
         <v>68</v>
       </c>
       <c r="B11" s="18"/>
@@ -1764,44 +1679,52 @@
       <c r="A12" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B12" s="32" t="s">
+      <c r="B12" s="35" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="26"/>
+      <c r="C12" s="32" t="s">
+        <v>156</v>
+      </c>
       <c r="D12" s="18"/>
     </row>
     <row r="13" spans="1:4" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B13" s="32" t="s">
+      <c r="B13" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="26"/>
+      <c r="C13" s="32" t="s">
+        <v>36</v>
+      </c>
       <c r="D13" s="18"/>
     </row>
     <row r="14" spans="1:4" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B14" s="32" t="s">
+      <c r="B14" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="26"/>
+      <c r="C14" s="32" t="s">
+        <v>36</v>
+      </c>
       <c r="D14" s="18"/>
     </row>
     <row r="15" spans="1:4" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B15" s="32" t="s">
+      <c r="B15" s="35" t="s">
         <v>57</v>
       </c>
-      <c r="C15" s="26"/>
+      <c r="C15" s="32" t="s">
+        <v>32</v>
+      </c>
       <c r="D15" s="18"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="21" t="s">
         <v>69</v>
       </c>
       <c r="B17" s="18"/>
@@ -1809,7 +1732,7 @@
       <c r="D17" s="18"/>
     </row>
     <row r="18" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="27" t="s">
+      <c r="A18" s="28" t="s">
         <v>70</v>
       </c>
       <c r="B18" s="18"/>
@@ -1851,7 +1774,9 @@
       <c r="B21" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="4"/>
+      <c r="C21" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D21" s="4"/>
     </row>
     <row r="22" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
@@ -1861,7 +1786,9 @@
       <c r="B22" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="C22" s="4"/>
+      <c r="C22" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D22" s="4"/>
     </row>
     <row r="23" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
@@ -1871,11 +1798,13 @@
       <c r="B23" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="C23" s="4"/>
+      <c r="C23" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D23" s="4"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="25" t="s">
+      <c r="A24" s="31" t="s">
         <v>71</v>
       </c>
       <c r="B24" s="18"/>
@@ -1886,11 +1815,11 @@
       <c r="A25" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B25" s="32" t="s">
+      <c r="B25" s="35" t="s">
         <v>54</v>
       </c>
-      <c r="C25" s="26" t="s">
-        <v>113</v>
+      <c r="C25" s="32" t="s">
+        <v>112</v>
       </c>
       <c r="D25" s="18"/>
     </row>
@@ -1898,10 +1827,10 @@
       <c r="A26" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B26" s="32" t="s">
+      <c r="B26" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="C26" s="31" t="s">
+      <c r="C26" s="34" t="s">
         <v>36</v>
       </c>
       <c r="D26" s="18"/>
@@ -1910,10 +1839,10 @@
       <c r="A27" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B27" s="32" t="s">
+      <c r="B27" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="C27" s="31" t="s">
+      <c r="C27" s="34" t="s">
         <v>36</v>
       </c>
       <c r="D27" s="18"/>
@@ -1922,26 +1851,16 @@
       <c r="A28" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B28" s="32" t="s">
+      <c r="B28" s="35" t="s">
         <v>57</v>
       </c>
-      <c r="C28" s="31" t="s">
-        <v>101</v>
+      <c r="C28" s="32" t="s">
+        <v>32</v>
       </c>
       <c r="D28" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="B15"/>
-    <mergeCell ref="B26"/>
-    <mergeCell ref="B28"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="B27"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="C26:D26"/>
@@ -1958,9 +1877,18 @@
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="C14:D14"/>
     <mergeCell ref="B14"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="B15"/>
+    <mergeCell ref="B26"/>
+    <mergeCell ref="B28"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="B27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1977,7 +1905,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>72</v>
       </c>
       <c r="B1" s="18"/>
@@ -1985,7 +1913,7 @@
       <c r="D1" s="18"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>39</v>
       </c>
       <c r="B2" s="18"/>
@@ -1993,7 +1921,7 @@
       <c r="D2" s="18"/>
     </row>
     <row r="3" spans="1:4" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="30" t="s">
         <v>73</v>
       </c>
       <c r="B3" s="18"/>
@@ -2001,7 +1929,7 @@
       <c r="D3" s="18"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
         <v>74</v>
       </c>
       <c r="B5" s="18"/>
@@ -2009,7 +1937,7 @@
       <c r="D5" s="18"/>
     </row>
     <row r="6" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="28" t="s">
         <v>75</v>
       </c>
       <c r="B6" s="18"/>
@@ -2020,11 +1948,11 @@
       <c r="A7" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="34"/>
-      <c r="D7" s="35"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="27"/>
     </row>
     <row r="8" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
@@ -2034,7 +1962,7 @@
         <v>48</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -2046,7 +1974,7 @@
         <v>49</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D9" s="4"/>
     </row>
@@ -2063,7 +1991,7 @@
       <c r="D10" s="4"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="31" t="s">
         <v>76</v>
       </c>
       <c r="B11" s="18"/>
@@ -2074,11 +2002,11 @@
       <c r="A12" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B12" s="32" t="s">
+      <c r="B12" s="35" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="26" t="s">
-        <v>114</v>
+      <c r="C12" s="32" t="s">
+        <v>113</v>
       </c>
       <c r="D12" s="18"/>
     </row>
@@ -2086,11 +2014,11 @@
       <c r="A13" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B13" s="32" t="s">
+      <c r="B13" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="26" t="s">
-        <v>115</v>
+      <c r="C13" s="32" t="s">
+        <v>114</v>
       </c>
       <c r="D13" s="18"/>
     </row>
@@ -2098,11 +2026,11 @@
       <c r="A14" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B14" s="32" t="s">
+      <c r="B14" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="26" t="s">
-        <v>116</v>
+      <c r="C14" s="32" t="s">
+        <v>115</v>
       </c>
       <c r="D14" s="18"/>
     </row>
@@ -2110,16 +2038,23 @@
       <c r="A15" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B15" s="32" t="s">
+      <c r="B15" s="35" t="s">
         <v>57</v>
       </c>
-      <c r="C15" s="26" t="s">
-        <v>117</v>
+      <c r="C15" s="32" t="s">
+        <v>116</v>
       </c>
       <c r="D15" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="B14"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="B15"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="B13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A6:D6"/>
@@ -2128,13 +2063,6 @@
     <mergeCell ref="A11:D11"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="B7:D7"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="B14"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="B15"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="B13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2153,7 +2081,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>77</v>
       </c>
       <c r="B1" s="18"/>
@@ -2161,7 +2089,7 @@
       <c r="D1" s="18"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>39</v>
       </c>
       <c r="B2" s="18"/>
@@ -2169,7 +2097,7 @@
       <c r="D2" s="18"/>
     </row>
     <row r="3" spans="1:4" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="30" t="s">
         <v>78</v>
       </c>
       <c r="B3" s="18"/>
@@ -2177,7 +2105,7 @@
       <c r="D3" s="18"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
         <v>79</v>
       </c>
       <c r="B5" s="18"/>
@@ -2185,7 +2113,7 @@
       <c r="D5" s="18"/>
     </row>
     <row r="6" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="28" t="s">
         <v>80</v>
       </c>
       <c r="B6" s="18"/>
@@ -2196,11 +2124,11 @@
       <c r="A7" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="34"/>
-      <c r="D7" s="35"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="27"/>
     </row>
     <row r="8" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
@@ -2210,7 +2138,7 @@
         <v>48</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -2221,7 +2149,9 @@
       <c r="B9" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="4"/>
+      <c r="C9" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D9" s="4"/>
     </row>
     <row r="10" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
@@ -2235,7 +2165,7 @@
       <c r="D10" s="4"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="31" t="s">
         <v>81</v>
       </c>
       <c r="B11" s="18"/>
@@ -2246,11 +2176,11 @@
       <c r="A12" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B12" s="32" t="s">
+      <c r="B12" s="35" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="26" t="s">
-        <v>118</v>
+      <c r="C12" s="32" t="s">
+        <v>117</v>
       </c>
       <c r="D12" s="18"/>
     </row>
@@ -2258,11 +2188,11 @@
       <c r="A13" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B13" s="32" t="s">
+      <c r="B13" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="26" t="s">
-        <v>119</v>
+      <c r="C13" s="32" t="s">
+        <v>118</v>
       </c>
       <c r="D13" s="18"/>
     </row>
@@ -2270,10 +2200,10 @@
       <c r="A14" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B14" s="32" t="s">
+      <c r="B14" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="31" t="s">
+      <c r="C14" s="34" t="s">
         <v>36</v>
       </c>
       <c r="D14" s="18"/>
@@ -2282,16 +2212,23 @@
       <c r="A15" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B15" s="32" t="s">
+      <c r="B15" s="35" t="s">
         <v>57</v>
       </c>
-      <c r="C15" s="26" t="s">
-        <v>120</v>
+      <c r="C15" s="32" t="s">
+        <v>119</v>
       </c>
       <c r="D15" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="B14"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="B15"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="B13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A6:D6"/>
@@ -2300,13 +2237,6 @@
     <mergeCell ref="A11:D11"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="B7:D7"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="B14"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="B15"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="B13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2325,21 +2255,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>82</v>
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="20" t="s">
         <v>83</v>
       </c>
       <c r="B2" s="18"/>
       <c r="C2" s="18"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="21" t="s">
         <v>84</v>
       </c>
       <c r="B4" s="18"/>
@@ -2353,7 +2283,7 @@
         <v>85</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
@@ -2364,7 +2294,7 @@
         <v>86</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
@@ -2375,7 +2305,7 @@
         <v>87</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
@@ -2386,7 +2316,7 @@
         <v>89</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
@@ -2397,11 +2327,11 @@
         <v>91</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="21" t="s">
         <v>92</v>
       </c>
       <c r="B11" s="18"/>
@@ -2415,7 +2345,7 @@
         <v>93</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
@@ -2448,7 +2378,7 @@
         <v>96</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
@@ -2470,7 +2400,7 @@
         <v>99</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -2499,7 +2429,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>38</v>
       </c>
       <c r="B1" s="18"/>
@@ -2507,7 +2437,7 @@
       <c r="D1" s="18"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>39</v>
       </c>
       <c r="B2" s="18"/>
@@ -2515,7 +2445,7 @@
       <c r="D2" s="18"/>
     </row>
     <row r="3" spans="1:4" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="30" t="s">
         <v>40</v>
       </c>
       <c r="B3" s="18"/>
@@ -2523,7 +2453,7 @@
       <c r="D3" s="18"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
         <v>41</v>
       </c>
       <c r="B5" s="18"/>
@@ -2531,7 +2461,7 @@
       <c r="D5" s="18"/>
     </row>
     <row r="6" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="28" t="s">
         <v>42</v>
       </c>
       <c r="B6" s="18"/>
@@ -2542,18 +2472,18 @@
       <c r="A7" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="34"/>
-      <c r="D7" s="35"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="27"/>
     </row>
     <row r="8" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
         <v>24</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -2565,7 +2495,9 @@
       <c r="B9" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="4"/>
+      <c r="C9" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D9" s="4"/>
     </row>
     <row r="10" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
@@ -2575,11 +2507,13 @@
       <c r="B10" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="4"/>
+      <c r="C10" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D10" s="4"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="31" t="s">
         <v>52</v>
       </c>
       <c r="B11" s="18"/>
@@ -2593,8 +2527,8 @@
       <c r="B12" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="26" t="s">
-        <v>131</v>
+      <c r="C12" s="32" t="s">
+        <v>130</v>
       </c>
       <c r="D12" s="18"/>
     </row>
@@ -2605,8 +2539,8 @@
       <c r="B13" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="26" t="s">
-        <v>130</v>
+      <c r="C13" s="32" t="s">
+        <v>129</v>
       </c>
       <c r="D13" s="18"/>
     </row>
@@ -2617,7 +2551,7 @@
       <c r="B14" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="26" t="s">
+      <c r="C14" s="32" t="s">
         <v>36</v>
       </c>
       <c r="D14" s="18"/>
@@ -2629,13 +2563,13 @@
       <c r="B15" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="C15" s="26" t="s">
+      <c r="C15" s="32" t="s">
         <v>32</v>
       </c>
       <c r="D15" s="18"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="21" t="s">
         <v>58</v>
       </c>
       <c r="B17" s="18"/>
@@ -2643,7 +2577,7 @@
       <c r="D17" s="18"/>
     </row>
     <row r="18" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="27" t="s">
+      <c r="A18" s="28" t="s">
         <v>59</v>
       </c>
       <c r="B18" s="18"/>
@@ -2654,11 +2588,11 @@
       <c r="A19" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B19" s="33" t="s">
+      <c r="B19" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="34"/>
-      <c r="D19" s="35"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="27"/>
     </row>
     <row r="20" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="13" t="s">
@@ -2681,7 +2615,9 @@
       <c r="B21" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="4"/>
+      <c r="C21" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D21" s="4"/>
     </row>
     <row r="22" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
@@ -2691,7 +2627,9 @@
       <c r="B22" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="C22" s="4"/>
+      <c r="C22" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D22" s="4"/>
     </row>
     <row r="23" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
@@ -2701,11 +2639,13 @@
       <c r="B23" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="C23" s="4"/>
+      <c r="C23" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D23" s="4"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="25" t="s">
+      <c r="A24" s="31" t="s">
         <v>60</v>
       </c>
       <c r="B24" s="18"/>
@@ -2719,8 +2659,8 @@
       <c r="B25" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C25" s="26" t="s">
-        <v>132</v>
+      <c r="C25" s="32" t="s">
+        <v>131</v>
       </c>
       <c r="D25" s="18"/>
     </row>
@@ -2731,7 +2671,7 @@
       <c r="B26" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="C26" s="26" t="s">
+      <c r="C26" s="32" t="s">
         <v>36</v>
       </c>
       <c r="D26" s="18"/>
@@ -2743,7 +2683,7 @@
       <c r="B27" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C27" s="26" t="s">
+      <c r="C27" s="32" t="s">
         <v>36</v>
       </c>
       <c r="D27" s="18"/>
@@ -2755,13 +2695,18 @@
       <c r="B28" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="C28" s="26" t="s">
+      <c r="C28" s="32" t="s">
         <v>32</v>
       </c>
       <c r="D28" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="C28:D28"/>
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="A18:D18"/>
     <mergeCell ref="A1:D1"/>
@@ -2776,11 +2721,6 @@
     <mergeCell ref="C14:D14"/>
     <mergeCell ref="C15:D15"/>
     <mergeCell ref="A17:D17"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C28:D28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2799,7 +2739,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>61</v>
       </c>
       <c r="B1" s="18"/>
@@ -2807,7 +2747,7 @@
       <c r="D1" s="18"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>39</v>
       </c>
       <c r="B2" s="18"/>
@@ -2815,15 +2755,15 @@
       <c r="D2" s="18"/>
     </row>
     <row r="3" spans="1:4" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="29" t="s">
-        <v>110</v>
+      <c r="A3" s="30" t="s">
+        <v>109</v>
       </c>
       <c r="B3" s="18"/>
       <c r="C3" s="18"/>
       <c r="D3" s="18"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
         <v>62</v>
       </c>
       <c r="B5" s="18"/>
@@ -2831,7 +2771,7 @@
       <c r="D5" s="18"/>
     </row>
     <row r="6" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="28" t="s">
         <v>63</v>
       </c>
       <c r="B6" s="18"/>
@@ -2842,18 +2782,18 @@
       <c r="A7" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="34"/>
-      <c r="D7" s="35"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="27"/>
     </row>
     <row r="8" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
         <v>24</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -2865,7 +2805,9 @@
       <c r="B9" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="4"/>
+      <c r="C9" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D9" s="4"/>
     </row>
     <row r="10" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
@@ -2875,11 +2817,13 @@
       <c r="B10" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="4"/>
+      <c r="C10" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D10" s="4"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="31" t="s">
         <v>64</v>
       </c>
       <c r="B11" s="18"/>
@@ -2893,8 +2837,8 @@
       <c r="B12" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="26" t="s">
-        <v>133</v>
+      <c r="C12" s="32" t="s">
+        <v>132</v>
       </c>
       <c r="D12" s="18"/>
     </row>
@@ -2905,7 +2849,7 @@
       <c r="B13" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="26" t="s">
+      <c r="C13" s="32" t="s">
         <v>36</v>
       </c>
       <c r="D13" s="18"/>
@@ -2917,7 +2861,7 @@
       <c r="B14" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="26" t="s">
+      <c r="C14" s="32" t="s">
         <v>36</v>
       </c>
       <c r="D14" s="18"/>
@@ -2929,7 +2873,7 @@
       <c r="B15" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="C15" s="26" t="s">
+      <c r="C15" s="32" t="s">
         <v>32</v>
       </c>
       <c r="D15" s="18"/>
@@ -2965,7 +2909,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>65</v>
       </c>
       <c r="B1" s="18"/>
@@ -2973,7 +2917,7 @@
       <c r="D1" s="18"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>39</v>
       </c>
       <c r="B2" s="18"/>
@@ -2981,7 +2925,7 @@
       <c r="D2" s="18"/>
     </row>
     <row r="3" spans="1:4" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="30" t="s">
+      <c r="A3" s="33" t="s">
         <v>100</v>
       </c>
       <c r="B3" s="18"/>
@@ -2989,7 +2933,7 @@
       <c r="D3" s="18"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
         <v>66</v>
       </c>
       <c r="B5" s="18"/>
@@ -2997,7 +2941,7 @@
       <c r="D5" s="18"/>
     </row>
     <row r="6" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="28" t="s">
         <v>67</v>
       </c>
       <c r="B6" s="18"/>
@@ -3008,20 +2952,18 @@
       <c r="A7" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="11"/>
-      <c r="D7" s="12" t="s">
-        <v>36</v>
-      </c>
+      <c r="C7" s="26"/>
+      <c r="D7" s="27"/>
     </row>
     <row r="8" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
         <v>24</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -3033,7 +2975,9 @@
       <c r="B9" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="4"/>
+      <c r="C9" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D9" s="4"/>
     </row>
     <row r="10" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
@@ -3043,11 +2987,13 @@
       <c r="B10" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="4"/>
+      <c r="C10" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D10" s="4"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="31" t="s">
         <v>68</v>
       </c>
       <c r="B11" s="18"/>
@@ -3061,8 +3007,8 @@
       <c r="B12" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="26" t="s">
-        <v>134</v>
+      <c r="C12" s="32" t="s">
+        <v>133</v>
       </c>
       <c r="D12" s="18"/>
     </row>
@@ -3073,7 +3019,7 @@
       <c r="B13" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="26" t="s">
+      <c r="C13" s="32" t="s">
         <v>36</v>
       </c>
       <c r="D13" s="18"/>
@@ -3085,7 +3031,7 @@
       <c r="B14" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="26" t="s">
+      <c r="C14" s="32" t="s">
         <v>36</v>
       </c>
       <c r="D14" s="18"/>
@@ -3097,13 +3043,13 @@
       <c r="B15" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="C15" s="26" t="s">
+      <c r="C15" s="32" t="s">
         <v>32</v>
       </c>
       <c r="D15" s="18"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="21" t="s">
         <v>69</v>
       </c>
       <c r="B17" s="18"/>
@@ -3111,7 +3057,7 @@
       <c r="D17" s="18"/>
     </row>
     <row r="18" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="27" t="s">
+      <c r="A18" s="28" t="s">
         <v>70</v>
       </c>
       <c r="B18" s="18"/>
@@ -3122,11 +3068,11 @@
       <c r="A19" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B19" s="33" t="s">
+      <c r="B19" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="34"/>
-      <c r="D19" s="35"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="27"/>
     </row>
     <row r="20" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="13" t="s">
@@ -3149,7 +3095,9 @@
       <c r="B21" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="4"/>
+      <c r="C21" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D21" s="4"/>
     </row>
     <row r="22" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
@@ -3159,7 +3107,9 @@
       <c r="B22" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="C22" s="4"/>
+      <c r="C22" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D22" s="4"/>
     </row>
     <row r="23" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
@@ -3169,11 +3119,13 @@
       <c r="B23" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="C23" s="4"/>
+      <c r="C23" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D23" s="4"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="25" t="s">
+      <c r="A24" s="31" t="s">
         <v>71</v>
       </c>
       <c r="B24" s="18"/>
@@ -3187,8 +3139,8 @@
       <c r="B25" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C25" s="26" t="s">
-        <v>135</v>
+      <c r="C25" s="32" t="s">
+        <v>134</v>
       </c>
       <c r="D25" s="18"/>
     </row>
@@ -3199,7 +3151,7 @@
       <c r="B26" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="C26" s="26" t="s">
+      <c r="C26" s="32" t="s">
         <v>36</v>
       </c>
       <c r="D26" s="18"/>
@@ -3211,7 +3163,7 @@
       <c r="B27" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C27" s="26" t="s">
+      <c r="C27" s="32" t="s">
         <v>36</v>
       </c>
       <c r="D27" s="18"/>
@@ -3223,13 +3175,18 @@
       <c r="B28" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="C28" s="26" t="s">
+      <c r="C28" s="32" t="s">
         <v>32</v>
       </c>
       <c r="D28" s="18"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="19">
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="C28:D28"/>
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="A18:D18"/>
     <mergeCell ref="A1:D1"/>
@@ -3243,14 +3200,9 @@
     <mergeCell ref="C14:D14"/>
     <mergeCell ref="C15:D15"/>
     <mergeCell ref="A17:D17"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="B7:D7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3267,7 +3219,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>72</v>
       </c>
       <c r="B1" s="18"/>
@@ -3275,7 +3227,7 @@
       <c r="D1" s="18"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>39</v>
       </c>
       <c r="B2" s="18"/>
@@ -3283,7 +3235,7 @@
       <c r="D2" s="18"/>
     </row>
     <row r="3" spans="1:4" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="30" t="s">
         <v>73</v>
       </c>
       <c r="B3" s="18"/>
@@ -3291,7 +3243,7 @@
       <c r="D3" s="18"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
         <v>74</v>
       </c>
       <c r="B5" s="18"/>
@@ -3299,7 +3251,7 @@
       <c r="D5" s="18"/>
     </row>
     <row r="6" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="28" t="s">
         <v>75</v>
       </c>
       <c r="B6" s="18"/>
@@ -3310,18 +3262,18 @@
       <c r="A7" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="34"/>
-      <c r="D7" s="35"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="27"/>
     </row>
     <row r="8" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
         <v>24</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C8" s="15"/>
       <c r="D8" s="4"/>
@@ -3333,7 +3285,9 @@
       <c r="B9" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="15"/>
+      <c r="C9" s="4" t="s">
+        <v>135</v>
+      </c>
       <c r="D9" s="4"/>
     </row>
     <row r="10" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
@@ -3349,7 +3303,7 @@
       <c r="D10" s="4"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="31" t="s">
         <v>76</v>
       </c>
       <c r="B11" s="18"/>
@@ -3363,8 +3317,8 @@
       <c r="B12" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="26" t="s">
-        <v>136</v>
+      <c r="C12" s="32" t="s">
+        <v>135</v>
       </c>
       <c r="D12" s="18"/>
     </row>
@@ -3375,8 +3329,8 @@
       <c r="B13" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="26" t="s">
-        <v>137</v>
+      <c r="C13" s="32" t="s">
+        <v>136</v>
       </c>
       <c r="D13" s="18"/>
     </row>
@@ -3387,8 +3341,8 @@
       <c r="B14" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="26" t="s">
-        <v>138</v>
+      <c r="C14" s="32" t="s">
+        <v>137</v>
       </c>
       <c r="D14" s="18"/>
     </row>
@@ -3399,8 +3353,8 @@
       <c r="B15" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="C15" s="26" t="s">
-        <v>139</v>
+      <c r="C15" s="32" t="s">
+        <v>138</v>
       </c>
       <c r="D15" s="18"/>
     </row>
@@ -3435,7 +3389,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>77</v>
       </c>
       <c r="B1" s="18"/>
@@ -3443,7 +3397,7 @@
       <c r="D1" s="18"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>39</v>
       </c>
       <c r="B2" s="18"/>
@@ -3451,7 +3405,7 @@
       <c r="D2" s="18"/>
     </row>
     <row r="3" spans="1:4" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="30" t="s">
         <v>78</v>
       </c>
       <c r="B3" s="18"/>
@@ -3459,7 +3413,7 @@
       <c r="D3" s="18"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
         <v>79</v>
       </c>
       <c r="B5" s="18"/>
@@ -3467,7 +3421,7 @@
       <c r="D5" s="18"/>
     </row>
     <row r="6" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="28" t="s">
         <v>80</v>
       </c>
       <c r="B6" s="18"/>
@@ -3478,18 +3432,18 @@
       <c r="A7" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="34"/>
-      <c r="D7" s="35"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="27"/>
     </row>
     <row r="8" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
         <v>24</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C8" s="15"/>
       <c r="D8" s="4"/>
@@ -3501,7 +3455,9 @@
       <c r="B9" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="4"/>
+      <c r="C9" s="4" t="s">
+        <v>155</v>
+      </c>
       <c r="D9" s="4"/>
     </row>
     <row r="10" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
@@ -3511,11 +3467,13 @@
       <c r="B10" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="4"/>
+      <c r="C10" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D10" s="4"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="31" t="s">
         <v>81</v>
       </c>
       <c r="B11" s="18"/>
@@ -3529,8 +3487,8 @@
       <c r="B12" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="26" t="s">
-        <v>140</v>
+      <c r="C12" s="32" t="s">
+        <v>139</v>
       </c>
       <c r="D12" s="18"/>
     </row>
@@ -3541,7 +3499,7 @@
       <c r="B13" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="26" t="s">
+      <c r="C13" s="32" t="s">
         <v>36</v>
       </c>
       <c r="D13" s="18"/>
@@ -3553,7 +3511,7 @@
       <c r="B14" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="26" t="s">
+      <c r="C14" s="32" t="s">
         <v>36</v>
       </c>
       <c r="D14" s="18"/>
@@ -3565,7 +3523,7 @@
       <c r="B15" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="C15" s="26" t="s">
+      <c r="C15" s="32" t="s">
         <v>32</v>
       </c>
       <c r="D15" s="18"/>
@@ -3601,21 +3559,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="28" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>82</v>
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
     </row>
     <row r="2" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="20" t="s">
         <v>83</v>
       </c>
       <c r="B2" s="18"/>
       <c r="C2" s="18"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="21" t="s">
         <v>84</v>
       </c>
       <c r="B4" s="18"/>
@@ -3629,7 +3587,7 @@
         <v>85</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
@@ -3640,7 +3598,7 @@
         <v>86</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
@@ -3651,7 +3609,7 @@
         <v>87</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
@@ -3662,7 +3620,7 @@
         <v>89</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
@@ -3673,11 +3631,11 @@
         <v>91</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="21" t="s">
         <v>92</v>
       </c>
       <c r="B11" s="18"/>
@@ -3691,7 +3649,7 @@
         <v>93</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
@@ -3702,7 +3660,7 @@
         <v>94</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
@@ -3713,7 +3671,7 @@
         <v>95</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
@@ -3724,7 +3682,7 @@
         <v>96</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
@@ -3735,7 +3693,7 @@
         <v>97</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
@@ -3746,7 +3704,7 @@
         <v>99</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -3775,7 +3733,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="18"/>
@@ -3783,15 +3741,15 @@
       <c r="D1" s="18"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="24" t="s">
-        <v>125</v>
+      <c r="A2" s="20" t="s">
+        <v>124</v>
       </c>
       <c r="B2" s="18"/>
       <c r="C2" s="18"/>
       <c r="D2" s="18"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="21" t="s">
         <v>1</v>
       </c>
       <c r="B4" s="18"/>
@@ -3819,7 +3777,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -3827,19 +3785,19 @@
         <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B9" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="22" t="s">
+      <c r="A10" s="21" t="s">
         <v>7</v>
       </c>
       <c r="B10" s="18"/>
@@ -3847,7 +3805,7 @@
       <c r="D10" s="18"/>
     </row>
     <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="17" t="s">
         <v>8</v>
       </c>
       <c r="B11" s="18"/>
@@ -3855,7 +3813,7 @@
       <c r="D11" s="18"/>
     </row>
     <row r="12" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="17" t="s">
         <v>9</v>
       </c>
       <c r="B12" s="18"/>
@@ -3863,7 +3821,7 @@
       <c r="D12" s="18"/>
     </row>
     <row r="13" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="17" t="s">
         <v>10</v>
       </c>
       <c r="B13" s="18"/>
@@ -3871,7 +3829,7 @@
       <c r="D13" s="18"/>
     </row>
     <row r="14" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="21" t="s">
+      <c r="A14" s="17" t="s">
         <v>11</v>
       </c>
       <c r="B14" s="18"/>
@@ -3879,7 +3837,7 @@
       <c r="D14" s="18"/>
     </row>
     <row r="15" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="21" t="s">
+      <c r="A15" s="17" t="s">
         <v>12</v>
       </c>
       <c r="B15" s="18"/>
@@ -3887,7 +3845,7 @@
       <c r="D15" s="18"/>
     </row>
     <row r="16" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="21" t="s">
+      <c r="A16" s="17" t="s">
         <v>13</v>
       </c>
       <c r="B16" s="18"/>
@@ -3895,7 +3853,7 @@
       <c r="D16" s="18"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="21" t="s">
         <v>14</v>
       </c>
       <c r="B18" s="18"/>
@@ -3987,7 +3945,7 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="22" t="s">
+      <c r="A26" s="21" t="s">
         <v>31</v>
       </c>
       <c r="B26" s="18"/>
@@ -3998,7 +3956,7 @@
       <c r="A27" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B27" s="17" t="s">
+      <c r="B27" s="22" t="s">
         <v>33</v>
       </c>
       <c r="C27" s="18"/>
@@ -4008,7 +3966,7 @@
       <c r="A28" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B28" s="19" t="s">
+      <c r="B28" s="23" t="s">
         <v>35</v>
       </c>
       <c r="C28" s="18"/>
@@ -4018,7 +3976,7 @@
       <c r="A29" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="B29" s="20" t="s">
+      <c r="B29" s="24" t="s">
         <v>37</v>
       </c>
       <c r="C29" s="18"/>
@@ -4061,7 +4019,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>38</v>
       </c>
       <c r="B1" s="18"/>
@@ -4069,7 +4027,7 @@
       <c r="D1" s="18"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>39</v>
       </c>
       <c r="B2" s="18"/>
@@ -4077,7 +4035,7 @@
       <c r="D2" s="18"/>
     </row>
     <row r="3" spans="1:4" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="30" t="s">
         <v>40</v>
       </c>
       <c r="B3" s="18"/>
@@ -4085,7 +4043,7 @@
       <c r="D3" s="18"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
         <v>41</v>
       </c>
       <c r="B5" s="18"/>
@@ -4093,7 +4051,7 @@
       <c r="D5" s="18"/>
     </row>
     <row r="6" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="28" t="s">
         <v>42</v>
       </c>
       <c r="B6" s="18"/>
@@ -4104,11 +4062,11 @@
       <c r="A7" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="34"/>
-      <c r="D7" s="35"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="27"/>
     </row>
     <row r="8" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
@@ -4127,7 +4085,9 @@
       <c r="B9" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="4"/>
+      <c r="C9" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D9" s="4"/>
     </row>
     <row r="10" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
@@ -4137,11 +4097,13 @@
       <c r="B10" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="4"/>
+      <c r="C10" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D10" s="4"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="31" t="s">
         <v>52</v>
       </c>
       <c r="B11" s="18"/>
@@ -4152,11 +4114,11 @@
       <c r="A12" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B12" s="32" t="s">
+      <c r="B12" s="35" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="26" t="s">
-        <v>107</v>
+      <c r="C12" s="32" t="s">
+        <v>106</v>
       </c>
       <c r="D12" s="18"/>
     </row>
@@ -4164,10 +4126,10 @@
       <c r="A13" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B13" s="32" t="s">
+      <c r="B13" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="31" t="s">
+      <c r="C13" s="34" t="s">
         <v>36</v>
       </c>
       <c r="D13" s="18"/>
@@ -4176,11 +4138,11 @@
       <c r="A14" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B14" s="32" t="s">
+      <c r="B14" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="26" t="s">
-        <v>108</v>
+      <c r="C14" s="32" t="s">
+        <v>107</v>
       </c>
       <c r="D14" s="18"/>
     </row>
@@ -4188,16 +4150,16 @@
       <c r="A15" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B15" s="32" t="s">
+      <c r="B15" s="35" t="s">
         <v>57</v>
       </c>
-      <c r="C15" s="31" t="s">
+      <c r="C15" s="34" t="s">
         <v>32</v>
       </c>
       <c r="D15" s="18"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="21" t="s">
         <v>58</v>
       </c>
       <c r="B17" s="18"/>
@@ -4205,7 +4167,7 @@
       <c r="D17" s="18"/>
     </row>
     <row r="18" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="27" t="s">
+      <c r="A18" s="28" t="s">
         <v>59</v>
       </c>
       <c r="B18" s="18"/>
@@ -4216,11 +4178,11 @@
       <c r="A19" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B19" s="33" t="s">
+      <c r="B19" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="34"/>
-      <c r="D19" s="35"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="27"/>
     </row>
     <row r="20" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="13" t="s">
@@ -4267,7 +4229,7 @@
       <c r="D23" s="4"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="25" t="s">
+      <c r="A24" s="31" t="s">
         <v>60</v>
       </c>
       <c r="B24" s="18"/>
@@ -4278,11 +4240,11 @@
       <c r="A25" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B25" s="32" t="s">
+      <c r="B25" s="35" t="s">
         <v>54</v>
       </c>
-      <c r="C25" s="26" t="s">
-        <v>127</v>
+      <c r="C25" s="32" t="s">
+        <v>126</v>
       </c>
       <c r="D25" s="18"/>
     </row>
@@ -4290,10 +4252,10 @@
       <c r="A26" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B26" s="32" t="s">
+      <c r="B26" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="C26" s="31" t="s">
+      <c r="C26" s="34" t="s">
         <v>36</v>
       </c>
       <c r="D26" s="18"/>
@@ -4302,11 +4264,11 @@
       <c r="A27" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B27" s="32" t="s">
+      <c r="B27" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="C27" s="26" t="s">
-        <v>109</v>
+      <c r="C27" s="32" t="s">
+        <v>108</v>
       </c>
       <c r="D27" s="18"/>
     </row>
@@ -4314,27 +4276,16 @@
       <c r="A28" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B28" s="32" t="s">
+      <c r="B28" s="35" t="s">
         <v>57</v>
       </c>
-      <c r="C28" s="31" t="s">
+      <c r="C28" s="34" t="s">
         <v>32</v>
       </c>
       <c r="D28" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="B15"/>
-    <mergeCell ref="B26"/>
-    <mergeCell ref="B28"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="B27"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="C26:D26"/>
@@ -4351,6 +4302,17 @@
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="C14:D14"/>
     <mergeCell ref="B14"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="B15"/>
+    <mergeCell ref="B26"/>
+    <mergeCell ref="B28"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="B27"/>
+    <mergeCell ref="B19:D19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>